<commit_message>
ANACONDA ENVIREMENT SETUP COMPLETED 3 DATA SETS CLEANED AND REVIEWED BY PANDAS IN JUPYTER NOTEBOOK
</commit_message>
<xml_diff>
--- a/DATA_SETS/q3-2.xlsx
+++ b/DATA_SETS/q3-2.xlsx
@@ -1,34 +1,94 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\farha\KRMU\GitHub\SEM-2-MINOR_PROJECT\DATA_SETS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED8675C-79F6-4334-BECE-1E104F99D3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dept_Fines_V2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dept_Fines_V2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Total_Borrows</t>
+  </si>
+  <si>
+    <t>Late_Returns</t>
+  </si>
+  <si>
+    <t>Total_Fines</t>
+  </si>
+  <si>
+    <t>Max_Fine</t>
+  </si>
+  <si>
+    <t>Min_Fine</t>
+  </si>
+  <si>
+    <t>Avg_Fine</t>
+  </si>
+  <si>
+    <t>Computer Science</t>
+  </si>
+  <si>
+    <t>Mechanical</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Civil</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>Arts</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>Law</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +106,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,300 +412,353 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="17.4609375" customWidth="1"/>
+    <col min="2" max="2" width="17.07421875" customWidth="1"/>
+    <col min="3" max="3" width="14.765625" customWidth="1"/>
+    <col min="4" max="4" width="12.23046875" customWidth="1"/>
+    <col min="5" max="5" width="11.07421875" customWidth="1"/>
+    <col min="6" max="6" width="9.3828125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Total_Borrows</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Late_Returns</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Total_Fines</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Max_Fine</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Min_Fine</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Avg_Fine</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Computer Science</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1">
         <v>571</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="1">
         <v>75</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="1">
         <v>3375</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="1">
         <v>184</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="1">
         <v>11</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="1">
         <v>45</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
         <v>414</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="1">
         <v>97</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="1">
         <v>4753</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="1">
         <v>108</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="1">
         <v>20</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="1">
         <v>49</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Electrical</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1">
         <v>545</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="1">
         <v>93</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="1">
         <v>2697</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="1">
         <v>181</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="1">
         <v>5</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="1">
         <v>29</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Civil</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1">
         <v>577</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="1">
         <v>89</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="1">
         <v>3560</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="1">
         <v>160</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="1">
         <v>12</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1">
         <v>527</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="1">
         <v>75</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="1">
         <v>2700</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="1">
         <v>116</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="1">
         <v>13</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="1">
         <v>36</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Arts</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1">
         <v>526</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="1">
         <v>77</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="1">
         <v>2464</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="1">
         <v>92</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="1">
         <v>16</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Science</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1">
         <v>393</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="1">
         <v>55</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="1">
         <v>2365</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1">
         <v>117</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="1">
         <v>13</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="1">
         <v>43</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Law</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="1">
         <v>334</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="1">
         <v>50</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="1">
         <v>1000</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="1">
         <v>171</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="1">
         <v>16</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1">
         <v>374</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="1">
         <v>52</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="1">
         <v>1196</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="1">
         <v>98</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="1">
         <v>17</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="1">
         <v>23</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1">
         <v>502</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="1">
         <v>84</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="1">
         <v>2352</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="1">
         <v>119</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="1">
         <v>10</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="1">
         <v>28</v>
       </c>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>